<commit_message>
fixed bug with configuration id
</commit_message>
<xml_diff>
--- a/Excel/test_output_spreadsheet.xlsx
+++ b/Excel/test_output_spreadsheet.xlsx
@@ -766,6 +766,42 @@
           <t>Baseline sweep - thrust at 6.5kN</t>
         </is>
       </c>
+      <c r="P4" t="n">
+        <v>4.016240282636565</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>26.88185800588363</v>
+      </c>
+      <c r="R4" t="n">
+        <v>3025.904364423432</v>
+      </c>
+      <c r="S4" t="n">
+        <v>3464.904364423432</v>
+      </c>
+      <c r="T4" t="n">
+        <v>235.2726541527136</v>
+      </c>
+      <c r="U4" t="n">
+        <v>65.18209090636971</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.7018742830875535</v>
+      </c>
+      <c r="W4" t="n">
+        <v>27.68161269043629</v>
+      </c>
+      <c r="X4" t="n">
+        <v>139.3431557033481</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>4.006235360503569</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>4.006235360503569</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>30045.20570535101</v>
+      </c>
     </row>
     <row r="5">
       <c r="C5" t="inlineStr">
@@ -895,6 +931,42 @@
         <is>
           <t>trajectory</t>
         </is>
+      </c>
+      <c r="P6" t="n">
+        <v>4.016538750579962</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>30.17597592103646</v>
+      </c>
+      <c r="R6" t="n">
+        <v>3119.731178807244</v>
+      </c>
+      <c r="S6" t="n">
+        <v>3558.731178807244</v>
+      </c>
+      <c r="T6" t="n">
+        <v>246.4317075421846</v>
+      </c>
+      <c r="U6" t="n">
+        <v>65.17999279123549</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.73434125174361</v>
+      </c>
+      <c r="W6" t="n">
+        <v>27.3536451073077</v>
+      </c>
+      <c r="X6" t="n">
+        <v>141.5391071267147</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>4.00626076801247</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>4.00626076801247</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>33269.2153188353</v>
       </c>
     </row>
     <row r="8">

</xml_diff>